<commit_message>
actualizacion final a la autoevaluacion
</commit_message>
<xml_diff>
--- a/TP-01-Autoevaluacion.xlsx
+++ b/TP-01-Autoevaluacion.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Formulario de autoevaluación</t>
   </si>
@@ -178,9 +178,6 @@
   </si>
   <si>
     <t>En esta sección puede ingresar cualquier comentario que el grupo le parezca pertinente, relacionado con la autoevaluación</t>
-  </si>
-  <si>
-    <t>Axel no hizo nadaMENTIRA</t>
   </si>
 </sst>
 </file>
@@ -521,7 +518,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="24.88"/>
-    <col customWidth="1" min="2" max="2" width="89.63"/>
+    <col customWidth="1" min="2" max="2" width="90.75"/>
     <col customWidth="1" min="3" max="3" width="16.5"/>
     <col customWidth="1" min="4" max="4" width="19.63"/>
     <col customWidth="1" min="5" max="6" width="12.63"/>
@@ -613,8 +610,8 @@
       <c r="B9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="7">
-        <v>2.0</v>
+      <c r="C9" s="9">
+        <v>8.0</v>
       </c>
       <c r="D9" s="7"/>
       <c r="E9" s="8"/>
@@ -709,8 +706,8 @@
       <c r="B13" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="7">
-        <v>7.0</v>
+      <c r="C13" s="9">
+        <v>8.0</v>
       </c>
       <c r="D13" s="7"/>
       <c r="E13" s="8"/>
@@ -757,10 +754,10 @@
       <c r="B15" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="7">
-        <v>6.0</v>
-      </c>
-      <c r="D15" s="7"/>
+      <c r="C15" s="9">
+        <v>7.0</v>
+      </c>
+      <c r="D15" s="9"/>
       <c r="E15" s="8"/>
       <c r="F15" s="8"/>
       <c r="G15" s="8"/>
@@ -782,7 +779,7 @@
         <v>26</v>
       </c>
       <c r="C16" s="9">
-        <v>6.0</v>
+        <v>7.0</v>
       </c>
       <c r="D16" s="7"/>
       <c r="E16" s="8"/>
@@ -805,9 +802,7 @@
       <c r="B17" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="9" t="s">
-        <v>29</v>
-      </c>
+      <c r="C17" s="9"/>
       <c r="D17" s="7"/>
       <c r="E17" s="8"/>
       <c r="F17" s="8"/>

</xml_diff>